<commit_message>
Implement compareWithFigma web path in BajajFinservWebTest
Rework BajajFinservWebTest into a data-driven TestNG test that reads
Web-platform rows from the compare input Excel, checks full page or a
Locator-scoped region against the uploadToFigma baseline, and writes
Comparison Batch URL/Validation Status back with a pass/fail summary.
Extend FigmaRow/ExcelHelper with Platform/Locator/comparison columns,
add a matching compare-input template, and update docs to reflect
step 4a as implemented.
</commit_message>
<xml_diff>
--- a/figma-visual-testing/figma_baseline_input_template.xlsx
+++ b/figma-visual-testing/figma_baseline_input_template.xlsx
@@ -423,15 +423,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,25 +443,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>UAT/Prod URL</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>App URL / Screen Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Viewport</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
@@ -474,13 +480,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>https://uat.example.com/homepage</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -490,29 +501,59 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>https://uat.example.com/cards</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>cards-component</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>1280x1024</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>png</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/abc123XYZ/My-Project?node-id=11-222</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Home Screen</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>android-home-screen</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>